<commit_message>
Updated my F1 files
</commit_message>
<xml_diff>
--- a/data/Formula_1/F1_2026.xlsx
+++ b/data/Formula_1/F1_2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vyan\Documents\GitHub\Formula_1\data\Formula_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11895F56-DCB2-47C8-AF33-282C42F93266}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{541C0894-32E2-418B-BECC-4D343A50CC50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="43095" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Schedule" sheetId="1" r:id="rId1"/>
@@ -1234,7 +1234,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1274,6 +1274,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2129,7 +2130,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="15" t="s">
         <v>205</v>
       </c>
     </row>
@@ -2200,7 +2201,7 @@
   <cols>
     <col min="1" max="1" width="4.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.88671875" customWidth="1"/>
     <col min="4" max="4" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>